<commit_message>
feat(hub): Adiciona modo de teste (F5+T) e corrige exclusão de UUIDs
</commit_message>
<xml_diff>
--- a/modelos/modelos_fluxo/XLSX - NNA - Expedientes Captados - 20260227.xlsx
+++ b/modelos/modelos_fluxo/XLSX - NNA - Expedientes Captados - 20260227.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B624140\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\B624140\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{00ABC22E-4BF5-4134-BF32-9AA14E444A57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7DE5092-99E8-48DB-89C4-40EF38FF3C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26327,7 +26327,7 @@
         <v>1510</v>
       </c>
       <c r="N197" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O197" t="s">
         <v>44</v>
@@ -26419,7 +26419,7 @@
         <v>1519</v>
       </c>
       <c r="N198" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O198" t="s">
         <v>44</v>
@@ -26511,7 +26511,7 @@
         <v>1527</v>
       </c>
       <c r="N199" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O199" t="s">
         <v>44</v>
@@ -26603,7 +26603,7 @@
         <v>1536</v>
       </c>
       <c r="N200" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O200" t="s">
         <v>44</v>
@@ -26695,7 +26695,7 @@
         <v>1545</v>
       </c>
       <c r="N201" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O201" t="s">
         <v>44</v>
@@ -26787,7 +26787,7 @@
         <v>1552</v>
       </c>
       <c r="N202" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O202" t="s">
         <v>44</v>
@@ -26971,7 +26971,7 @@
         <v>1570</v>
       </c>
       <c r="N204" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O204" t="s">
         <v>44</v>
@@ -27063,7 +27063,7 @@
         <v>1578</v>
       </c>
       <c r="N205" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O205" t="s">
         <v>44</v>
@@ -27155,7 +27155,7 @@
         <v>1587</v>
       </c>
       <c r="N206" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O206" t="s">
         <v>44</v>
@@ -27247,7 +27247,7 @@
         <v>1595</v>
       </c>
       <c r="N207" t="s">
-        <v>218</v>
+        <v>1302</v>
       </c>
       <c r="O207" t="s">
         <v>44</v>

</xml_diff>